<commit_message>
Update courses from spreadsheet
</commit_message>
<xml_diff>
--- a/co_courses.xlsx
+++ b/co_courses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/camcrabtree/Desktop/colorado_map_clone/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E3AAAC-A082-3545-B0D5-CE683ADEBD2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE954CC6-60E9-5543-A2EA-E37C92B099F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="702">
   <si>
     <t>Course</t>
   </si>
@@ -2130,10 +2130,6 @@
   </si>
   <si>
     <t>Bond</t>
-  </si>
-  <si>
-    <t>39.89846
-</t>
   </si>
   <si>
     <t>https://www.instagram.com/p/DWtge96ByI2/</t>
@@ -2534,7 +2530,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2754,19 +2750,13 @@
     <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -9385,14 +9375,14 @@
       <c r="E201" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F201" s="82" t="s">
-        <v>701</v>
+      <c r="F201" s="80" t="s">
+        <v>700</v>
       </c>
       <c r="G201" s="19">
         <v>-105.067701</v>
       </c>
       <c r="H201" s="13" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="I201" s="24">
         <v>45363</v>
@@ -9581,14 +9571,14 @@
       <c r="E207" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="F207" s="85">
+      <c r="F207" s="83">
         <v>39.352437000000002</v>
       </c>
       <c r="G207" s="19">
         <v>-104.857772</v>
       </c>
-      <c r="H207" s="84" t="s">
-        <v>702</v>
+      <c r="H207" s="82" t="s">
+        <v>701</v>
       </c>
       <c r="I207" s="53">
         <v>44759</v>
@@ -10571,27 +10561,27 @@
       <c r="A239" s="38" t="s">
         <v>695</v>
       </c>
-      <c r="B239" s="77" t="s">
+      <c r="B239" s="12" t="s">
         <v>696</v>
       </c>
-      <c r="C239" s="78" t="s">
+      <c r="C239" s="35" t="s">
         <v>697</v>
       </c>
-      <c r="D239" s="78" t="s">
+      <c r="D239" s="35" t="s">
         <v>29</v>
       </c>
       <c r="E239" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="F239" s="83" t="s">
-        <v>698</v>
+      <c r="F239" s="81">
+        <v>39.89846</v>
       </c>
       <c r="G239" s="19">
         <v>-106.712484</v>
       </c>
-      <c r="H239" s="79"/>
-      <c r="I239" s="80"/>
-      <c r="J239" s="81"/>
+      <c r="H239" s="77"/>
+      <c r="I239" s="78"/>
+      <c r="J239" s="79"/>
     </row>
     <row r="240" spans="1:10" ht="22.5" customHeight="1">
       <c r="A240" s="15" t="s">
@@ -11921,8 +11911,8 @@
       <c r="G282" s="19">
         <v>-105.1336</v>
       </c>
-      <c r="H282" s="84" t="s">
-        <v>699</v>
+      <c r="H282" s="82" t="s">
+        <v>698</v>
       </c>
       <c r="I282" s="53">
         <v>44672</v>

</xml_diff>